<commit_message>
added missionplans to repo
</commit_message>
<xml_diff>
--- a/messplan.xlsx
+++ b/messplan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexa\Desktop\Studium\Laufend\Mechatronik und Leistungselektronik Projekt VU\project_code\orbitalPropagatorComparison\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCDB6DBA-C083-4AAF-9DCB-A88C5237BAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF23D6B-A2F3-4C4F-B480-34A0D1F309BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="72">
   <si>
     <t>Satellite</t>
   </si>
@@ -239,6 +239,21 @@
   </si>
   <si>
     <t>12458U</t>
+  </si>
+  <si>
+    <t>probleme mit der belichtungszeit</t>
+  </si>
+  <si>
+    <t>still some troubles, but needs checking, debris might be too dark simply</t>
+  </si>
+  <si>
+    <t>nice track</t>
+  </si>
+  <si>
+    <t>satellite only at beginning, moves out of field</t>
+  </si>
+  <si>
+    <t>satellite moves out of frame</t>
   </si>
 </sst>
 </file>
@@ -261,7 +276,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -292,6 +307,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -305,14 +344,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -975,7 +1019,7 @@
     <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="40.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="59.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -1029,7 +1073,10 @@
       <c r="F3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -1051,7 +1098,10 @@
       <c r="F4" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="5"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="8" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="5" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1073,7 +1123,10 @@
       <c r="F5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="5"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -1095,7 +1148,10 @@
       <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="8" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="7" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -1117,7 +1173,10 @@
       <c r="F7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="5"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="1" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1139,7 +1198,10 @@
       <c r="F8" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="5"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="8" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="9" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1161,7 +1223,10 @@
       <c r="F9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -1183,7 +1248,10 @@
       <c r="F10" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="5"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="8" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="11" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
@@ -1227,9 +1295,8 @@
       <c r="F12" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>59</v>
       </c>
@@ -1270,8 +1337,9 @@
       <c r="F14" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G14" s="11"/>
+    </row>
+    <row r="15" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>63</v>
       </c>
@@ -1291,6 +1359,7 @@
       <c r="F15" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="G15" s="11"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">

</xml_diff>